<commit_message>
update to species reference list
</commit_message>
<xml_diff>
--- a/data/metadata/GLNPO Species List.xlsx
+++ b/data/metadata/GLNPO Species List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51703220-E92E-4E69-A3DF-909E407565DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B972DD55-061A-4576-9F54-34994DDCD642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11280" xr2:uid="{B7CFF889-1C41-4D14-95B5-EC43053AFCDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7CFF889-1C41-4D14-95B5-EC43053AFCDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Zoops" sheetId="1" r:id="rId1"/>
@@ -1886,16 +1886,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA087434-B657-4664-8F46-47D5BD24A1FF}">
   <dimension ref="A1:E103"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" style="11" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="29.5546875" style="11" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" style="11" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
         <v>219</v>
       </c>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
@@ -1925,7 +1925,7 @@
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="17" t="s">
         <v>3</v>
       </c>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>7</v>
       </c>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
         <v>9</v>
       </c>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="17" t="s">
         <v>11</v>
       </c>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
         <v>13</v>
       </c>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="17" t="s">
         <v>15</v>
       </c>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
         <v>17</v>
       </c>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
         <v>19</v>
       </c>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
         <v>21</v>
       </c>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
         <v>23</v>
       </c>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
         <v>26</v>
       </c>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
         <v>30</v>
       </c>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
         <v>32</v>
       </c>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
         <v>34</v>
       </c>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="E16" s="3"/>
     </row>
-    <row r="17" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
         <v>37</v>
       </c>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
         <v>39</v>
       </c>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
         <v>41</v>
       </c>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="17" t="s">
         <v>43</v>
       </c>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
         <v>45</v>
       </c>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="17" t="s">
         <v>47</v>
       </c>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="17" t="s">
         <v>49</v>
       </c>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="17" t="s">
         <v>51</v>
       </c>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="E24" s="3"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="17" t="s">
         <v>53</v>
       </c>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="17" t="s">
         <v>55</v>
       </c>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="17" t="s">
         <v>58</v>
       </c>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
         <v>60</v>
       </c>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="17" t="s">
         <v>63</v>
       </c>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="17" t="s">
         <v>65</v>
       </c>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A31" s="17" t="s">
         <v>67</v>
       </c>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="E31" s="3"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="17" t="s">
         <v>69</v>
       </c>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="E32" s="3"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="17" t="s">
         <v>71</v>
       </c>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="E33" s="3"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="17" t="s">
         <v>73</v>
       </c>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="E34" s="3"/>
     </row>
-    <row r="35" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="17" t="s">
         <v>75</v>
       </c>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="E35" s="3"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="17" t="s">
         <v>77</v>
       </c>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="E36" s="3"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="17" t="s">
         <v>79</v>
       </c>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="17" t="s">
         <v>81</v>
       </c>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="E38" s="3"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="17" t="s">
         <v>83</v>
       </c>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="E39" s="3"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="17" t="s">
         <v>85</v>
       </c>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="E40" s="3"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="17" t="s">
         <v>87</v>
       </c>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="17" t="s">
         <v>89</v>
       </c>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="E42" s="3"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="17" t="s">
         <v>91</v>
       </c>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="E43" s="3"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="17" t="s">
         <v>93</v>
       </c>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="17" t="s">
         <v>95</v>
       </c>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="17" t="s">
         <v>97</v>
       </c>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="17" t="s">
         <v>99</v>
       </c>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="E47" s="3"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="17" t="s">
         <v>101</v>
       </c>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="17" t="s">
         <v>103</v>
       </c>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="E49" s="3"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="17" t="s">
         <v>105</v>
       </c>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="E50" s="3"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
         <v>107</v>
       </c>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="E51" s="3"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="17" t="s">
         <v>110</v>
       </c>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="E52" s="3"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
         <v>112</v>
       </c>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="17" t="s">
         <v>114</v>
       </c>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="17" t="s">
         <v>116</v>
       </c>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="17" t="s">
         <v>118</v>
       </c>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="E56" s="3"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="17" t="s">
         <v>120</v>
       </c>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="E57" s="3"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="17" t="s">
         <v>122</v>
       </c>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="E58" s="3"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="17" t="s">
         <v>124</v>
       </c>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="E59" s="3"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="19" t="s">
         <v>126</v>
       </c>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="E60" s="3"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="17" t="s">
         <v>128</v>
       </c>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="E61" s="3"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="17" t="s">
         <v>130</v>
       </c>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="E62" s="3"/>
     </row>
-    <row r="63" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="17" t="s">
         <v>132</v>
       </c>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="E63" s="3"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="17" t="s">
         <v>134</v>
       </c>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="E64" s="3"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="17" t="s">
         <v>136</v>
       </c>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E65" s="3"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="17" t="s">
         <v>138</v>
       </c>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="E66" s="3"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="17" t="s">
         <v>140</v>
       </c>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="E67" s="3"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="17" t="s">
         <v>142</v>
       </c>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="E68" s="3"/>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="20" t="s">
         <v>144</v>
       </c>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="E69" s="3"/>
     </row>
-    <row r="70" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="17" t="s">
         <v>146</v>
       </c>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="E70" s="3"/>
     </row>
-    <row r="71" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="17" t="s">
         <v>148</v>
       </c>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="E71" s="3"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="17" t="s">
         <v>150</v>
       </c>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="E72" s="3"/>
     </row>
-    <row r="73" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A73" s="17" t="s">
         <v>152</v>
       </c>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="E73" s="3"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="17" t="s">
         <v>154</v>
       </c>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="17" t="s">
         <v>156</v>
       </c>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="E75" s="3"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="17" t="s">
         <v>158</v>
       </c>
@@ -3035,7 +3035,7 @@
       </c>
       <c r="E76" s="3"/>
     </row>
-    <row r="77" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A77" s="17" t="s">
         <v>160</v>
       </c>
@@ -3050,7 +3050,7 @@
       </c>
       <c r="E77" s="3"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="17" t="s">
         <v>162</v>
       </c>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="E78" s="3"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="17" t="s">
         <v>164</v>
       </c>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="E79" s="3"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="17" t="s">
         <v>166</v>
       </c>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="E80" s="3"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="17" t="s">
         <v>168</v>
       </c>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="E81" s="3"/>
     </row>
-    <row r="82" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A82" s="17" t="s">
         <v>170</v>
       </c>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="E82" s="3"/>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="17" t="s">
         <v>172</v>
       </c>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="E83" s="3"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="17" t="s">
         <v>174</v>
       </c>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="E84" s="3"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="17" t="s">
         <v>176</v>
       </c>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="E85" s="3"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="17" t="s">
         <v>178</v>
       </c>
@@ -3185,7 +3185,7 @@
       </c>
       <c r="E86" s="3"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="20" t="s">
         <v>181</v>
       </c>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="E87" s="3"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="17" t="s">
         <v>183</v>
       </c>
@@ -3211,7 +3211,7 @@
       <c r="D88" s="19"/>
       <c r="E88" s="3"/>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="17" t="s">
         <v>185</v>
       </c>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="17" t="s">
         <v>187</v>
       </c>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="17" t="s">
         <v>189</v>
       </c>
@@ -3256,7 +3256,7 @@
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="17" t="s">
         <v>191</v>
       </c>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="17" t="s">
         <v>193</v>
       </c>
@@ -3286,7 +3286,7 @@
       </c>
       <c r="E93" s="3"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="17" t="s">
         <v>195</v>
       </c>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="E94" s="3"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="17" t="s">
         <v>197</v>
       </c>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="E95" s="3"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="17" t="s">
         <v>199</v>
       </c>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="E96" s="3"/>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" s="17" t="s">
         <v>201</v>
       </c>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="E97" s="3"/>
     </row>
-    <row r="98" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A98" s="17" t="s">
         <v>203</v>
       </c>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="21" t="s">
         <v>205</v>
       </c>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="E99" s="3"/>
     </row>
-    <row r="100" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="17" t="s">
         <v>207</v>
       </c>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="E100" s="3"/>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" s="17" t="s">
         <v>209</v>
       </c>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="E101" s="4"/>
     </row>
-    <row r="102" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A102" s="17" t="s">
         <v>211</v>
       </c>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="E102" s="3"/>
     </row>
-    <row r="103" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A103" s="17" t="s">
         <v>213</v>
       </c>
@@ -3444,16 +3444,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB3ABFC-07F3-4D77-8DE4-4391782C47C5}">
   <dimension ref="A1:G111"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.85546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" style="11" customWidth="1"/>
+    <col min="1" max="1" width="28.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="11" customWidth="1"/>
     <col min="4" max="4" width="10" style="11" customWidth="1"/>
-    <col min="6" max="7" width="9.140625" customWidth="1"/>
+    <col min="6" max="7" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
         <v>219</v>
       </c>
@@ -3469,7 +3469,7 @@
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>222</v>
       </c>
@@ -3485,7 +3485,7 @@
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>225</v>
       </c>
@@ -3501,7 +3501,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>228</v>
       </c>
@@ -3517,7 +3517,7 @@
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>230</v>
       </c>
@@ -3533,7 +3533,7 @@
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>232</v>
       </c>
@@ -3549,7 +3549,7 @@
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>234</v>
       </c>
@@ -3565,7 +3565,7 @@
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>236</v>
       </c>
@@ -3581,7 +3581,7 @@
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>238</v>
       </c>
@@ -3597,7 +3597,7 @@
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>240</v>
       </c>
@@ -3613,7 +3613,7 @@
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>242</v>
       </c>
@@ -3629,7 +3629,7 @@
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>244</v>
       </c>
@@ -3645,7 +3645,7 @@
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>246</v>
       </c>
@@ -3661,7 +3661,7 @@
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>248</v>
       </c>
@@ -3677,7 +3677,7 @@
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>250</v>
       </c>
@@ -3693,7 +3693,7 @@
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>252</v>
       </c>
@@ -3709,7 +3709,7 @@
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>254</v>
       </c>
@@ -3725,7 +3725,7 @@
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>256</v>
       </c>
@@ -3741,7 +3741,7 @@
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
         <v>258</v>
       </c>
@@ -3757,7 +3757,7 @@
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>260</v>
       </c>
@@ -3773,7 +3773,7 @@
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>262</v>
       </c>
@@ -3789,7 +3789,7 @@
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
         <v>264</v>
       </c>
@@ -3805,7 +3805,7 @@
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
         <v>266</v>
       </c>
@@ -3821,7 +3821,7 @@
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
         <v>268</v>
       </c>
@@ -3837,7 +3837,7 @@
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
         <v>270</v>
       </c>
@@ -3853,7 +3853,7 @@
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>272</v>
       </c>
@@ -3869,7 +3869,7 @@
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="s">
         <v>274</v>
       </c>
@@ -3885,7 +3885,7 @@
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
         <v>276</v>
       </c>
@@ -3901,7 +3901,7 @@
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="10" t="s">
         <v>278</v>
       </c>
@@ -3917,7 +3917,7 @@
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
         <v>280</v>
       </c>
@@ -3933,7 +3933,7 @@
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
         <v>282</v>
       </c>
@@ -3949,7 +3949,7 @@
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="10" t="s">
         <v>284</v>
       </c>
@@ -3965,7 +3965,7 @@
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="10" t="s">
         <v>286</v>
       </c>
@@ -3981,7 +3981,7 @@
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="10" t="s">
         <v>288</v>
       </c>
@@ -3997,7 +3997,7 @@
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
         <v>290</v>
       </c>
@@ -4013,7 +4013,7 @@
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
         <v>292</v>
       </c>
@@ -4029,7 +4029,7 @@
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="10" t="s">
         <v>294</v>
       </c>
@@ -4045,7 +4045,7 @@
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="10" t="s">
         <v>296</v>
       </c>
@@ -4061,7 +4061,7 @@
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="10" t="s">
         <v>298</v>
       </c>
@@ -4077,7 +4077,7 @@
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="10" t="s">
         <v>300</v>
       </c>
@@ -4093,7 +4093,7 @@
       <c r="F40" s="6"/>
       <c r="G40" s="6"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
         <v>302</v>
       </c>
@@ -4109,7 +4109,7 @@
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
         <v>304</v>
       </c>
@@ -4125,7 +4125,7 @@
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="10" t="s">
         <v>306</v>
       </c>
@@ -4141,7 +4141,7 @@
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="10" t="s">
         <v>308</v>
       </c>
@@ -4157,7 +4157,7 @@
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="10" t="s">
         <v>310</v>
       </c>
@@ -4173,7 +4173,7 @@
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
         <v>312</v>
       </c>
@@ -4189,7 +4189,7 @@
       <c r="F46" s="6"/>
       <c r="G46" s="6"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
         <v>314</v>
       </c>
@@ -4205,7 +4205,7 @@
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
         <v>316</v>
       </c>
@@ -4221,7 +4221,7 @@
       <c r="F48" s="6"/>
       <c r="G48" s="6"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="10" t="s">
         <v>318</v>
       </c>
@@ -4237,7 +4237,7 @@
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="10" t="s">
         <v>320</v>
       </c>
@@ -4253,7 +4253,7 @@
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="10" t="s">
         <v>322</v>
       </c>
@@ -4269,7 +4269,7 @@
       <c r="F51" s="6"/>
       <c r="G51" s="6"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="10" t="s">
         <v>324</v>
       </c>
@@ -4285,7 +4285,7 @@
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="10" t="s">
         <v>326</v>
       </c>
@@ -4301,7 +4301,7 @@
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="10" t="s">
         <v>328</v>
       </c>
@@ -4317,7 +4317,7 @@
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="10" t="s">
         <v>330</v>
       </c>
@@ -4333,7 +4333,7 @@
       <c r="F55" s="6"/>
       <c r="G55" s="6"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="10" t="s">
         <v>332</v>
       </c>
@@ -4349,7 +4349,7 @@
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
         <v>334</v>
       </c>
@@ -4365,7 +4365,7 @@
       <c r="F57" s="6"/>
       <c r="G57" s="6"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="10" t="s">
         <v>336</v>
       </c>
@@ -4381,7 +4381,7 @@
       <c r="F58" s="6"/>
       <c r="G58" s="6"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="10" t="s">
         <v>338</v>
       </c>
@@ -4397,7 +4397,7 @@
       <c r="F59" s="6"/>
       <c r="G59" s="6"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="10" t="s">
         <v>340</v>
       </c>
@@ -4413,7 +4413,7 @@
       <c r="F60" s="6"/>
       <c r="G60" s="6"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="10" t="s">
         <v>342</v>
       </c>
@@ -4429,7 +4429,7 @@
       <c r="F61" s="6"/>
       <c r="G61" s="6"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="10" t="s">
         <v>344</v>
       </c>
@@ -4445,7 +4445,7 @@
       <c r="F62" s="6"/>
       <c r="G62" s="6"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="10" t="s">
         <v>346</v>
       </c>
@@ -4461,7 +4461,7 @@
       <c r="F63" s="6"/>
       <c r="G63" s="6"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="10" t="s">
         <v>348</v>
       </c>
@@ -4477,7 +4477,7 @@
       <c r="F64" s="6"/>
       <c r="G64" s="6"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="10" t="s">
         <v>350</v>
       </c>
@@ -4493,7 +4493,7 @@
       <c r="F65" s="6"/>
       <c r="G65" s="6"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="10" t="s">
         <v>352</v>
       </c>
@@ -4509,7 +4509,7 @@
       <c r="F66" s="6"/>
       <c r="G66" s="6"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="10" t="s">
         <v>354</v>
       </c>
@@ -4525,7 +4525,7 @@
       <c r="F67" s="6"/>
       <c r="G67" s="6"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="10" t="s">
         <v>356</v>
       </c>
@@ -4541,7 +4541,7 @@
       <c r="F68" s="6"/>
       <c r="G68" s="6"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="10" t="s">
         <v>358</v>
       </c>
@@ -4557,7 +4557,7 @@
       <c r="F69" s="6"/>
       <c r="G69" s="6"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="10" t="s">
         <v>360</v>
       </c>
@@ -4573,7 +4573,7 @@
       <c r="F70" s="6"/>
       <c r="G70" s="6"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="10" t="s">
         <v>362</v>
       </c>
@@ -4589,7 +4589,7 @@
       <c r="F71" s="6"/>
       <c r="G71" s="6"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="10" t="s">
         <v>364</v>
       </c>
@@ -4605,7 +4605,7 @@
       <c r="F72" s="6"/>
       <c r="G72" s="6"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="10" t="s">
         <v>366</v>
       </c>
@@ -4621,7 +4621,7 @@
       <c r="F73" s="6"/>
       <c r="G73" s="6"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="10" t="s">
         <v>368</v>
       </c>
@@ -4637,7 +4637,7 @@
       <c r="F74" s="6"/>
       <c r="G74" s="6"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="10" t="s">
         <v>370</v>
       </c>
@@ -4653,7 +4653,7 @@
       <c r="F75" s="6"/>
       <c r="G75" s="6"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="10" t="s">
         <v>372</v>
       </c>
@@ -4669,7 +4669,7 @@
       <c r="F76" s="6"/>
       <c r="G76" s="6"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="10" t="s">
         <v>374</v>
       </c>
@@ -4685,7 +4685,7 @@
       <c r="F77" s="6"/>
       <c r="G77" s="6"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="10" t="s">
         <v>376</v>
       </c>
@@ -4701,7 +4701,7 @@
       <c r="F78" s="6"/>
       <c r="G78" s="6"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="10" t="s">
         <v>378</v>
       </c>
@@ -4717,7 +4717,7 @@
       <c r="F79" s="6"/>
       <c r="G79" s="6"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="10" t="s">
         <v>380</v>
       </c>
@@ -4733,7 +4733,7 @@
       <c r="F80" s="6"/>
       <c r="G80" s="6"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" s="10" t="s">
         <v>382</v>
       </c>
@@ -4749,7 +4749,7 @@
       <c r="F81" s="6"/>
       <c r="G81" s="6"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="10" t="s">
         <v>384</v>
       </c>
@@ -4765,7 +4765,7 @@
       <c r="F82" s="6"/>
       <c r="G82" s="6"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="10" t="s">
         <v>386</v>
       </c>
@@ -4781,7 +4781,7 @@
       <c r="F83" s="6"/>
       <c r="G83" s="6"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="10" t="s">
         <v>388</v>
       </c>
@@ -4797,7 +4797,7 @@
       <c r="F84" s="6"/>
       <c r="G84" s="6"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="10" t="s">
         <v>390</v>
       </c>
@@ -4813,7 +4813,7 @@
       <c r="F85" s="6"/>
       <c r="G85" s="6"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="10" t="s">
         <v>392</v>
       </c>
@@ -4829,7 +4829,7 @@
       <c r="F86" s="6"/>
       <c r="G86" s="6"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="10" t="s">
         <v>394</v>
       </c>
@@ -4845,7 +4845,7 @@
       <c r="F87" s="6"/>
       <c r="G87" s="6"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="10" t="s">
         <v>396</v>
       </c>
@@ -4861,7 +4861,7 @@
       <c r="F88" s="6"/>
       <c r="G88" s="6"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" s="10" t="s">
         <v>398</v>
       </c>
@@ -4877,7 +4877,7 @@
       <c r="F89" s="6"/>
       <c r="G89" s="6"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="14" t="s">
         <v>400</v>
       </c>
@@ -4893,7 +4893,7 @@
       <c r="F90" s="8"/>
       <c r="G90" s="8"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" s="10" t="s">
         <v>402</v>
       </c>
@@ -4909,7 +4909,7 @@
       <c r="F91" s="6"/>
       <c r="G91" s="6"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="10" t="s">
         <v>404</v>
       </c>
@@ -4925,7 +4925,7 @@
       <c r="F92" s="6"/>
       <c r="G92" s="6"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" s="10" t="s">
         <v>406</v>
       </c>
@@ -4941,7 +4941,7 @@
       <c r="F93" s="6"/>
       <c r="G93" s="6"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" s="10" t="s">
         <v>408</v>
       </c>
@@ -4957,7 +4957,7 @@
       <c r="F94" s="6"/>
       <c r="G94" s="6"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" s="10" t="s">
         <v>408</v>
       </c>
@@ -4973,7 +4973,7 @@
       <c r="F95" s="6"/>
       <c r="G95" s="6"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" s="10" t="s">
         <v>410</v>
       </c>
@@ -4989,7 +4989,7 @@
       <c r="F96" s="6"/>
       <c r="G96" s="6"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" s="10" t="s">
         <v>412</v>
       </c>
@@ -5005,7 +5005,7 @@
       <c r="F97" s="6"/>
       <c r="G97" s="6"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" s="10" t="s">
         <v>414</v>
       </c>
@@ -5021,7 +5021,7 @@
       <c r="F98" s="6"/>
       <c r="G98" s="6"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" s="10" t="s">
         <v>416</v>
       </c>
@@ -5037,7 +5037,7 @@
       <c r="F99" s="6"/>
       <c r="G99" s="6"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" s="10" t="s">
         <v>418</v>
       </c>
@@ -5053,7 +5053,7 @@
       <c r="F100" s="6"/>
       <c r="G100" s="6"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" s="10" t="s">
         <v>420</v>
       </c>
@@ -5069,7 +5069,7 @@
       <c r="F101" s="6"/>
       <c r="G101" s="6"/>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102" s="10" t="s">
         <v>422</v>
       </c>
@@ -5085,7 +5085,7 @@
       <c r="F102" s="6"/>
       <c r="G102" s="6"/>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="10" t="s">
         <v>424</v>
       </c>
@@ -5101,7 +5101,7 @@
       <c r="F103" s="6"/>
       <c r="G103" s="6"/>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104" s="10" t="s">
         <v>426</v>
       </c>
@@ -5117,7 +5117,7 @@
       <c r="F104" s="6"/>
       <c r="G104" s="6"/>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105" s="10" t="s">
         <v>428</v>
       </c>
@@ -5133,7 +5133,7 @@
       <c r="F105" s="6"/>
       <c r="G105" s="6"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106" s="10" t="s">
         <v>430</v>
       </c>
@@ -5149,7 +5149,7 @@
       <c r="F106" s="6"/>
       <c r="G106" s="6"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107" s="10" t="s">
         <v>432</v>
       </c>
@@ -5165,7 +5165,7 @@
       <c r="F107" s="6"/>
       <c r="G107" s="6"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108" s="10" t="s">
         <v>434</v>
       </c>
@@ -5181,7 +5181,7 @@
       <c r="F108" s="6"/>
       <c r="G108" s="6"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109" s="10" t="s">
         <v>436</v>
       </c>
@@ -5197,7 +5197,7 @@
       <c r="F109" s="6"/>
       <c r="G109" s="6"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" s="10" t="s">
         <v>438</v>
       </c>
@@ -5213,7 +5213,7 @@
       <c r="F110" s="6"/>
       <c r="G110" s="6"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111" s="14" t="s">
         <v>440</v>
       </c>

</xml_diff>

<commit_message>
adjusting CYCIM to CYCIMM and CALIM to CYCIMM in Species reference list
</commit_message>
<xml_diff>
--- a/data/metadata/GLNPO Species List.xlsx
+++ b/data/metadata/GLNPO Species List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B972DD55-061A-4576-9F54-34994DDCD642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0652632-694B-4CB7-9146-EA8058C4EBC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7CFF889-1C41-4D14-95B5-EC43053AFCDF}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{B7CFF889-1C41-4D14-95B5-EC43053AFCDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Zoops" sheetId="1" r:id="rId1"/>
@@ -132,9 +132,6 @@
     <t>CAL</t>
   </si>
   <si>
-    <t>CALIM</t>
-  </si>
-  <si>
     <t>Camptocercus rectirostris</t>
   </si>
   <si>
@@ -216,9 +213,6 @@
     <t>CYCCOPE</t>
   </si>
   <si>
-    <t>CYCIM</t>
-  </si>
-  <si>
     <t>Cyclops strenuus</t>
   </si>
   <si>
@@ -318,9 +312,6 @@
     <t>DAPSP</t>
   </si>
   <si>
-    <t>Diaptomid copepodites</t>
-  </si>
-  <si>
     <t>DIACOPE</t>
   </si>
   <si>
@@ -1369,6 +1360,15 @@
   </si>
   <si>
     <t>SUBGROUP</t>
+  </si>
+  <si>
+    <t>Diaptomus copepodites</t>
+  </si>
+  <si>
+    <t>CALIMM</t>
+  </si>
+  <si>
+    <t>CYCIMM</t>
   </si>
 </sst>
 </file>
@@ -1885,6 +1885,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA087434-B657-4664-8F46-47D5BD24A1FF}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E103"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1897,20 +1898,20 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
@@ -1921,11 +1922,11 @@
         <v>2</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17" t="s">
         <v>3</v>
       </c>
@@ -1940,7 +1941,7 @@
       </c>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
         <v>7</v>
       </c>
@@ -1955,7 +1956,7 @@
       </c>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
         <v>9</v>
       </c>
@@ -1970,7 +1971,7 @@
       </c>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="17" t="s">
         <v>11</v>
       </c>
@@ -1985,7 +1986,7 @@
       </c>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
         <v>13</v>
       </c>
@@ -2000,7 +2001,7 @@
       </c>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="17" t="s">
         <v>15</v>
       </c>
@@ -2015,7 +2016,7 @@
       </c>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
         <v>17</v>
       </c>
@@ -2030,7 +2031,7 @@
       </c>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
         <v>19</v>
       </c>
@@ -2045,7 +2046,7 @@
       </c>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
         <v>21</v>
       </c>
@@ -2060,7 +2061,7 @@
       </c>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="17" t="s">
         <v>23</v>
       </c>
@@ -2075,7 +2076,7 @@
       </c>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
         <v>26</v>
       </c>
@@ -2083,19 +2084,19 @@
         <v>27</v>
       </c>
       <c r="C13" s="19" t="s">
+        <v>440</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="17" t="s">
+      <c r="B14" s="17" t="s">
         <v>30</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>31</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>6</v>
@@ -2105,12 +2106,12 @@
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>32</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>33</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>6</v>
@@ -2120,72 +2121,72 @@
       </c>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="C16" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="D16" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="17" t="s">
+      <c r="B17" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="C17" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="17" t="s">
+      <c r="B18" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="C18" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="E18" s="3"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
+      <c r="B19" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="C19" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="E19" s="3"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="17" t="s">
+      <c r="B20" s="17" t="s">
         <v>43</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>44</v>
       </c>
       <c r="C20" s="19" t="s">
         <v>25</v>
@@ -2195,12 +2196,12 @@
       </c>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="17" t="s">
         <v>45</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>46</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>6</v>
@@ -2210,12 +2211,12 @@
       </c>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="17" t="s">
         <v>47</v>
-      </c>
-      <c r="B22" s="17" t="s">
-        <v>48</v>
       </c>
       <c r="C22" s="19" t="s">
         <v>6</v>
@@ -2225,12 +2226,12 @@
       </c>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="17" t="s">
         <v>49</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>50</v>
       </c>
       <c r="C23" s="19" t="s">
         <v>6</v>
@@ -2240,12 +2241,12 @@
       </c>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="17" t="s">
         <v>51</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>52</v>
       </c>
       <c r="C24" s="19" t="s">
         <v>6</v>
@@ -2255,12 +2256,12 @@
       </c>
       <c r="E24" s="3"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="17" t="s">
         <v>53</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>54</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>6</v>
@@ -2272,295 +2273,295 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="C26" s="19" t="s">
+        <v>441</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="B27" s="17" t="s">
         <v>57</v>
-      </c>
-      <c r="D26" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E26" s="3"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>59</v>
       </c>
       <c r="C27" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="D28" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="19" t="s">
+      <c r="B29" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E28" s="3"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="17" t="s">
+      <c r="C29" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B30" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D29" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E29" s="3"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="17" t="s">
+      <c r="C30" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B31" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D30" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E30" s="3"/>
-    </row>
-    <row r="31" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A31" s="17" t="s">
+      <c r="C31" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B32" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="C31" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E31" s="3"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="17" t="s">
+      <c r="C32" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E32" s="3"/>
+    </row>
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B33" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D32" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E32" s="3"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="17" t="s">
+      <c r="C33" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D33" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E33" s="3"/>
+    </row>
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B34" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D33" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E33" s="3"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="17" t="s">
+      <c r="C34" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E34" s="3"/>
+    </row>
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B34" s="17" t="s">
+      <c r="B35" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D34" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E34" s="3"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="17" t="s">
+      <c r="C35" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D35" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E35" s="3"/>
+    </row>
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B36" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D35" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E35" s="3"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="17" t="s">
+      <c r="C36" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E36" s="3"/>
+    </row>
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="B36" s="17" t="s">
+      <c r="B37" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="C36" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D36" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E36" s="3"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="17" t="s">
+      <c r="C37" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D37" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E37" s="3"/>
+    </row>
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B38" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C37" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D37" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E37" s="3"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="17" t="s">
+      <c r="C38" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D38" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E38" s="3"/>
+    </row>
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="B39" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="C38" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D38" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E38" s="3"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="17" t="s">
+      <c r="C39" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D39" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E39" s="3"/>
+    </row>
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="B40" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C39" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D39" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E39" s="3"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="17" t="s">
+      <c r="C40" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D40" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E40" s="3"/>
+    </row>
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B41" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="C40" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D40" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E40" s="3"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="17" t="s">
+      <c r="C41" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D41" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E41" s="3"/>
+    </row>
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="B41" s="17" t="s">
+      <c r="B42" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C41" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D41" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E41" s="3"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="17" t="s">
+      <c r="C42" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D42" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="E42" s="3"/>
+    </row>
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="17" t="s">
+        <v>439</v>
+      </c>
+      <c r="B43" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="B42" s="17" t="s">
+      <c r="C43" s="19" t="s">
+        <v>440</v>
+      </c>
+      <c r="D43" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E43" s="3"/>
+    </row>
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C42" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="D42" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="E42" s="3"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="17" t="s">
+      <c r="B44" s="17" t="s">
         <v>91</v>
-      </c>
-      <c r="B43" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="C43" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D43" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E43" s="3"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>94</v>
       </c>
       <c r="C44" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="17" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C45" s="19" t="s">
         <v>6</v>
@@ -2570,12 +2571,12 @@
       </c>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="17" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C46" s="19" t="s">
         <v>6</v>
@@ -2585,102 +2586,102 @@
       </c>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C47" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E47" s="3"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="17" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C48" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D48" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>440</v>
+      </c>
+      <c r="D49" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E49" s="3"/>
+    </row>
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B50" s="17" t="s">
         <v>103</v>
-      </c>
-      <c r="B49" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D49" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E49" s="3"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="B50" s="17" t="s">
-        <v>106</v>
       </c>
       <c r="C50" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D50" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E50" s="3"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="B51" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C51" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="E51" s="3"/>
+    </row>
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="B51" s="17" t="s">
+      <c r="B52" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="C51" s="19" t="s">
+      <c r="C52" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D52" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="E52" s="3"/>
+    </row>
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="D51" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="E51" s="3"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A52" s="17" t="s">
+      <c r="B53" s="17" t="s">
         <v>110</v>
-      </c>
-      <c r="B52" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C52" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="D52" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="E52" s="3"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="B53" s="17" t="s">
-        <v>113</v>
       </c>
       <c r="C53" s="19" t="s">
         <v>6</v>
@@ -2690,12 +2691,12 @@
       </c>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="17" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C54" s="19" t="s">
         <v>6</v>
@@ -2705,102 +2706,102 @@
       </c>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="17" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C55" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D55" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="B56" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="C56" s="19" t="s">
+        <v>440</v>
+      </c>
+      <c r="D56" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E56" s="3"/>
+    </row>
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="B57" s="17" t="s">
         <v>118</v>
-      </c>
-      <c r="B56" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="C56" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D56" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E56" s="3"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A57" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="B57" s="17" t="s">
-        <v>121</v>
       </c>
       <c r="C57" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D57" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E57" s="3"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="B58" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="C58" s="19" t="s">
+        <v>441</v>
+      </c>
+      <c r="D58" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E58" s="3"/>
+    </row>
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B59" s="17" t="s">
         <v>122</v>
-      </c>
-      <c r="B58" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D58" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E58" s="3"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A59" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="B59" s="17" t="s">
-        <v>125</v>
       </c>
       <c r="C59" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D59" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E59" s="3"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="19" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C60" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D60" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E60" s="3"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="17" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B61" s="17" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C61" s="19" t="s">
         <v>6</v>
@@ -2810,57 +2811,57 @@
       </c>
       <c r="E61" s="3"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="17" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B62" s="17" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C62" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D62" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E62" s="3"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="B63" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="C63" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D63" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E63" s="3"/>
+    </row>
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="B64" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="B63" s="17" t="s">
+      <c r="C64" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D64" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="E64" s="3"/>
+    </row>
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="C63" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D63" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E63" s="3"/>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A64" s="17" t="s">
+      <c r="B65" s="17" t="s">
         <v>134</v>
-      </c>
-      <c r="B64" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="C64" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D64" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="E64" s="3"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A65" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="B65" s="17" t="s">
-        <v>137</v>
       </c>
       <c r="C65" s="19" t="s">
         <v>6</v>
@@ -2870,12 +2871,12 @@
       </c>
       <c r="E65" s="3"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="17" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B66" s="17" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C66" s="19" t="s">
         <v>6</v>
@@ -2885,12 +2886,12 @@
       </c>
       <c r="E66" s="3"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="17" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B67" s="17" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C67" s="19" t="s">
         <v>6</v>
@@ -2900,12 +2901,12 @@
       </c>
       <c r="E67" s="3"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="17" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C68" s="19" t="s">
         <v>6</v>
@@ -2915,12 +2916,12 @@
       </c>
       <c r="E68" s="3"/>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="20" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B69" s="20" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C69" s="19" t="s">
         <v>6</v>
@@ -2930,72 +2931,72 @@
       </c>
       <c r="E69" s="3"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="17" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C70" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D70" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E70" s="3"/>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="17" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B71" s="17" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C71" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D71" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E71" s="3"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="17" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B72" s="17" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C72" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D72" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E72" s="3"/>
     </row>
-    <row r="73" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="17" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B73" s="17" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C73" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D73" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E73" s="3"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="17" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B74" s="17" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C74" s="19" t="s">
         <v>25</v>
@@ -3005,12 +3006,12 @@
       </c>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="17" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B75" s="17" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C75" s="19" t="s">
         <v>6</v>
@@ -3020,12 +3021,12 @@
       </c>
       <c r="E75" s="3"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="17" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B76" s="17" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C76" s="19" t="s">
         <v>6</v>
@@ -3035,42 +3036,42 @@
       </c>
       <c r="E76" s="3"/>
     </row>
-    <row r="77" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="B77" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="C77" s="19" t="s">
+        <v>440</v>
+      </c>
+      <c r="D77" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E77" s="3"/>
+    </row>
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="B78" s="17" t="s">
         <v>160</v>
-      </c>
-      <c r="B77" s="17" t="s">
-        <v>161</v>
-      </c>
-      <c r="C77" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D77" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E77" s="3"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A78" s="17" t="s">
-        <v>162</v>
-      </c>
-      <c r="B78" s="17" t="s">
-        <v>163</v>
       </c>
       <c r="C78" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D78" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E78" s="3"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="17" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C79" s="19" t="s">
         <v>6</v>
@@ -3080,12 +3081,12 @@
       </c>
       <c r="E79" s="3"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="17" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B80" s="17" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C80" s="19" t="s">
         <v>6</v>
@@ -3095,72 +3096,72 @@
       </c>
       <c r="E80" s="3"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="17" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C81" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D81" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E81" s="3"/>
     </row>
-    <row r="82" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="B82" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="C82" s="19" t="s">
+        <v>441</v>
+      </c>
+      <c r="D82" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E82" s="3"/>
+    </row>
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="B83" s="17" t="s">
         <v>170</v>
-      </c>
-      <c r="B82" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="C82" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D82" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E82" s="3"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A83" s="17" t="s">
-        <v>172</v>
-      </c>
-      <c r="B83" s="17" t="s">
-        <v>173</v>
       </c>
       <c r="C83" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D83" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E83" s="3"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="17" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B84" s="17" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C84" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D84" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E84" s="3"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="17" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B85" s="17" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C85" s="19" t="s">
         <v>6</v>
@@ -3170,68 +3171,68 @@
       </c>
       <c r="E85" s="3"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="B86" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="C86" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="D86" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="E86" s="3"/>
+    </row>
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="20" t="s">
         <v>178</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B87" s="20" t="s">
         <v>179</v>
-      </c>
-      <c r="C86" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="D86" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="E86" s="3"/>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A87" s="20" t="s">
-        <v>181</v>
-      </c>
-      <c r="B87" s="20" t="s">
-        <v>182</v>
       </c>
       <c r="C87" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E87" s="3"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="17" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B88" s="17" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C88" s="19"/>
       <c r="D88" s="19"/>
       <c r="E88" s="3"/>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="17" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B89" s="17" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C89" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="17" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B90" s="17" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C90" s="19" t="s">
         <v>6</v>
@@ -3241,12 +3242,12 @@
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="17" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B91" s="17" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C91" s="19" t="s">
         <v>6</v>
@@ -3256,12 +3257,12 @@
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="17" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B92" s="17" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C92" s="19" t="s">
         <v>25</v>
@@ -3271,12 +3272,12 @@
       </c>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="17" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B93" s="17" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C93" s="19" t="s">
         <v>6</v>
@@ -3286,12 +3287,12 @@
       </c>
       <c r="E93" s="3"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="17" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B94" s="17" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C94" s="19" t="s">
         <v>6</v>
@@ -3301,42 +3302,42 @@
       </c>
       <c r="E94" s="3"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="17" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B95" s="17" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C95" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D95" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E95" s="3"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="B96" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="C96" s="19" t="s">
+        <v>440</v>
+      </c>
+      <c r="D96" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E96" s="3"/>
+    </row>
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="B97" s="17" t="s">
         <v>199</v>
-      </c>
-      <c r="B96" s="17" t="s">
-        <v>200</v>
-      </c>
-      <c r="C96" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D96" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E96" s="3"/>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A97" s="17" t="s">
-        <v>201</v>
-      </c>
-      <c r="B97" s="17" t="s">
-        <v>202</v>
       </c>
       <c r="C97" s="19" t="s">
         <v>6</v>
@@ -3346,97 +3347,104 @@
       </c>
       <c r="E97" s="3"/>
     </row>
-    <row r="98" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="17" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B98" s="17" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C98" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D98" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E98" s="3"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="21" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B99" s="20" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C99" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D99" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E99" s="3"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="17" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B100" s="17" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C100" s="19" t="s">
         <v>28</v>
       </c>
       <c r="D100" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E100" s="3"/>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="17" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B101" s="17" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C101" s="22" t="s">
         <v>2</v>
       </c>
       <c r="D101" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E101" s="4"/>
     </row>
-    <row r="102" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="B102" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="C102" s="19" t="s">
+        <v>441</v>
+      </c>
+      <c r="D102" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E102" s="3"/>
+    </row>
+    <row r="103" spans="1:5" ht="31.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="B103" s="17" t="s">
         <v>211</v>
-      </c>
-      <c r="B102" s="17" t="s">
-        <v>212</v>
-      </c>
-      <c r="C102" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D102" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E102" s="3"/>
-    </row>
-    <row r="103" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A103" s="17" t="s">
-        <v>213</v>
-      </c>
-      <c r="B103" s="17" t="s">
-        <v>214</v>
       </c>
       <c r="C103" s="19" t="s">
         <v>2</v>
       </c>
       <c r="D103" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E103" s="3"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D103" xr:uid="{FA087434-B657-4664-8F46-47D5BD24A1FF}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="CYCIM"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3455,1776 +3463,1776 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="10" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="10" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="10" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="10" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="10" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="10" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="10" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="10" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="6"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="10" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="10" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="10" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F46" s="6"/>
       <c r="G46" s="6"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="6"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="10" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="10" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="10" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="6"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="10" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="10" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="10" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="10" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F55" s="6"/>
       <c r="G55" s="6"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="10" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F57" s="6"/>
       <c r="G57" s="6"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="10" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F58" s="6"/>
       <c r="G58" s="6"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="10" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F59" s="6"/>
       <c r="G59" s="6"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="10" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F60" s="6"/>
       <c r="G60" s="6"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="10" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F61" s="6"/>
       <c r="G61" s="6"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="10" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="6"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="10" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F63" s="6"/>
       <c r="G63" s="6"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="10" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F64" s="6"/>
       <c r="G64" s="6"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="10" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F65" s="6"/>
       <c r="G65" s="6"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="10" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F66" s="6"/>
       <c r="G66" s="6"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="10" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="10" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F68" s="6"/>
       <c r="G68" s="6"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="10" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F69" s="6"/>
       <c r="G69" s="6"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="10" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F70" s="6"/>
       <c r="G70" s="6"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="10" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D71" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F71" s="6"/>
       <c r="G71" s="6"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="10" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D72" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F72" s="6"/>
       <c r="G72" s="6"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="10" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D73" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F73" s="6"/>
       <c r="G73" s="6"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="10" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F74" s="6"/>
       <c r="G74" s="6"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="10" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D75" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F75" s="6"/>
       <c r="G75" s="6"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="10" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F76" s="6"/>
       <c r="G76" s="6"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="10" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="C77" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D77" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F77" s="6"/>
       <c r="G77" s="6"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="10" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D78" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F78" s="6"/>
       <c r="G78" s="6"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="10" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D79" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F79" s="6"/>
       <c r="G79" s="6"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="10" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F80" s="6"/>
       <c r="G80" s="6"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" s="10" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F81" s="6"/>
       <c r="G81" s="6"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="10" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F82" s="6"/>
       <c r="G82" s="6"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="10" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="C83" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D83" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F83" s="6"/>
       <c r="G83" s="6"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="10" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="C84" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D84" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F84" s="6"/>
       <c r="G84" s="6"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="10" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="C85" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D85" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F85" s="6"/>
       <c r="G85" s="6"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="10" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C86" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D86" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F86" s="6"/>
       <c r="G86" s="6"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="10" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="C87" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D87" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F87" s="6"/>
       <c r="G87" s="6"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="10" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D88" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F88" s="6"/>
       <c r="G88" s="6"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" s="10" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D89" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F89" s="6"/>
       <c r="G89" s="6"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="14" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="B90" s="14" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D90" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F90" s="8"/>
       <c r="G90" s="8"/>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" s="10" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D91" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F91" s="6"/>
       <c r="G91" s="6"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="10" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C92" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D92" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F92" s="6"/>
       <c r="G92" s="6"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" s="10" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="C93" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D93" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F93" s="6"/>
       <c r="G93" s="6"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" s="10" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D94" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F94" s="6"/>
       <c r="G94" s="6"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" s="10" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D95" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F95" s="6"/>
       <c r="G95" s="6"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" s="10" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="C96" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D96" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F96" s="6"/>
       <c r="G96" s="6"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" s="10" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C97" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D97" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F97" s="6"/>
       <c r="G97" s="6"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" s="10" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D98" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F98" s="6"/>
       <c r="G98" s="6"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" s="10" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D99" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F99" s="6"/>
       <c r="G99" s="6"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" s="10" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B100" s="10" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="C100" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D100" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F100" s="6"/>
       <c r="G100" s="6"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" s="10" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="B101" s="10" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C101" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D101" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F101" s="6"/>
       <c r="G101" s="6"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102" s="10" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="B102" s="10" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C102" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D102" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F102" s="6"/>
       <c r="G102" s="6"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="10" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="B103" s="10" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C103" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D103" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F103" s="6"/>
       <c r="G103" s="6"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104" s="10" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="B104" s="10" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="C104" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D104" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F104" s="6"/>
       <c r="G104" s="6"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105" s="10" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="B105" s="10" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C105" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D105" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F105" s="6"/>
       <c r="G105" s="6"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106" s="10" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="B106" s="10" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="C106" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D106" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F106" s="6"/>
       <c r="G106" s="6"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107" s="10" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="C107" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D107" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F107" s="6"/>
       <c r="G107" s="6"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108" s="10" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="C108" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D108" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F108" s="6"/>
       <c r="G108" s="6"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109" s="10" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="B109" s="10" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C109" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D109" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F109" s="6"/>
       <c r="G109" s="6"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" s="10" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="B110" s="10" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="C110" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D110" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F110" s="6"/>
       <c r="G110" s="6"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111" s="14" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="B111" s="14" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="C111" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D111" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F111" s="8"/>
       <c r="G111" s="8"/>

</xml_diff>